<commit_message>
BeseLaTeng and Malieketseng inputs
</commit_message>
<xml_diff>
--- a/uGridNet Start Packet/uGrid_Input.xlsx
+++ b/uGridNet Start Packet/uGrid_Input.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mostation/Projects/1PWR/uGrid_uGridNet/uGridNet Start Packet/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D2B0ADF-1277-AA4C-8C3E-E046D261414F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57BF7063-E794-0A49-A26D-04BF1CB781F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" tabRatio="500" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -355,7 +355,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="4">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -370,6 +370,18 @@
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="9.8000000000000007"/>
+      <color rgb="FFA9B7C6"/>
+      <name val="JetBrains Mono"/>
+      <family val="3"/>
     </font>
   </fonts>
   <fills count="2">
@@ -401,7 +413,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -416,6 +428,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -744,7 +758,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:O2"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.5" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.5" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="7.6640625" customWidth="1"/>
     <col min="2" max="2" width="7.1640625" customWidth="1"/>
@@ -761,7 +775,7 @@
     <col min="15" max="15" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:15">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -808,7 +822,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:15">
       <c r="A2">
         <v>50</v>
       </c>
@@ -865,7 +879,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:AM3"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.5" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.5" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="7.1640625" customWidth="1"/>
     <col min="2" max="5" width="5" customWidth="1"/>
@@ -905,7 +919,7 @@
     <col min="39" max="39" width="18.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:39" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:39">
       <c r="A1" t="s">
         <v>16</v>
       </c>
@@ -1024,7 +1038,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="2" spans="1:39" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:39">
       <c r="A2">
         <v>15</v>
       </c>
@@ -1145,7 +1159,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="3" spans="1:39" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:39">
       <c r="O3" t="s">
         <v>55</v>
       </c>
@@ -1162,7 +1176,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:D2"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.5" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.5" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="5.6640625" customWidth="1"/>
     <col min="2" max="2" width="14.5" customWidth="1"/>
@@ -1170,7 +1184,7 @@
     <col min="4" max="4" width="11" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:4">
       <c r="A1" t="s">
         <v>56</v>
       </c>
@@ -1184,7 +1198,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:4">
       <c r="A2">
         <v>1</v>
       </c>
@@ -1207,9 +1221,9 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:K2"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.5" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.5" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:11">
       <c r="A1" t="s">
         <v>60</v>
       </c>
@@ -1244,7 +1258,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:11">
       <c r="A2">
         <v>2005</v>
       </c>
@@ -1287,8 +1301,8 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:N2"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.5" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:N3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.5" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="13.33203125" customWidth="1"/>
     <col min="2" max="2" width="13.83203125" customWidth="1"/>
@@ -1304,7 +1318,7 @@
     <col min="13" max="13" width="7.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:14">
       <c r="A1" t="s">
         <v>71</v>
       </c>
@@ -1348,7 +1362,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:14" ht="16">
       <c r="A2">
         <v>1</v>
       </c>
@@ -1367,11 +1381,11 @@
       <c r="F2">
         <v>500</v>
       </c>
-      <c r="G2">
-        <v>-29.178957</v>
-      </c>
-      <c r="H2">
-        <v>27.590275999999999</v>
+      <c r="G2" s="6">
+        <v>-29.873325000000001</v>
+      </c>
+      <c r="H2" s="6">
+        <v>28.61674</v>
       </c>
       <c r="I2">
         <v>0.34343958370448102</v>
@@ -1393,6 +1407,9 @@
       <c r="N2">
         <v>1</v>
       </c>
+    </row>
+    <row r="3" spans="1:14">
+      <c r="D3" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.51180555555555496" footer="0.51180555555555496"/>
@@ -1403,13 +1420,13 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:B15"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="40.1640625" style="1" customWidth="1"/>
     <col min="2" max="2" width="12.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:2">
       <c r="A1" s="2" t="s">
         <v>85</v>
       </c>
@@ -1417,7 +1434,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:2">
       <c r="A2" s="1" t="s">
         <v>87</v>
       </c>
@@ -1425,7 +1442,7 @@
         <v>4843.6050704225399</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:2">
       <c r="A3" s="1" t="s">
         <v>88</v>
       </c>
@@ -1433,7 +1450,7 @@
         <v>2052.7914788732401</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:2">
       <c r="A4" s="1" t="s">
         <v>89</v>
       </c>
@@ -1441,7 +1458,7 @@
         <v>193.130345070423</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:2">
       <c r="A5" s="1" t="s">
         <v>90</v>
       </c>
@@ -1449,7 +1466,7 @@
         <v>305.027464788732</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:2">
       <c r="A6" s="1" t="s">
         <v>91</v>
       </c>
@@ -1457,7 +1474,7 @@
         <v>430.23233098591601</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:2">
       <c r="A7" s="1" t="s">
         <v>92</v>
       </c>
@@ -1465,7 +1482,7 @@
         <v>193.33028169014099</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:2">
       <c r="A8" s="1" t="s">
         <v>93</v>
       </c>
@@ -1473,7 +1490,7 @@
         <v>52.491533802816903</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:2">
       <c r="A9" s="1" t="s">
         <v>94</v>
       </c>
@@ -1481,7 +1498,7 @@
         <v>80.771533802816904</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:2">
       <c r="A10" s="1" t="s">
         <v>95</v>
       </c>
@@ -1489,7 +1506,7 @@
         <v>114.961392957746</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:2">
       <c r="A11" s="1" t="s">
         <v>96</v>
       </c>
@@ -1497,7 +1514,7 @@
         <v>81.239999999999995</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:2">
       <c r="A12" s="1" t="s">
         <v>97</v>
       </c>
@@ -1505,7 +1522,7 @@
         <v>2.46</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:2">
       <c r="A13" s="1" t="s">
         <v>98</v>
       </c>
@@ -1513,7 +1530,7 @@
         <v>2.04</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:2">
       <c r="A14" s="1" t="s">
         <v>99</v>
       </c>
@@ -1521,7 +1538,7 @@
         <v>2.04</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:2">
       <c r="A15" s="1" t="s">
         <v>100</v>
       </c>

</xml_diff>